<commit_message>
chore: update xlxs template
</commit_message>
<xml_diff>
--- a/app/routes/generate-reports/.server/workbooks/report.xlsx
+++ b/app/routes/generate-reports/.server/workbooks/report.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Лист 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Лист 1'!$A$9:$U$276</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Лист 1'!$A$9:$U$277</definedName>
   </definedNames>
   <calcPr calcId="152511" iterateDelta="1E-4"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1518" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1523" uniqueCount="391">
   <si>
     <t>Приложение  к распоряжению №___ от________</t>
   </si>
@@ -1197,6 +1197,9 @@
   </si>
   <si>
     <t>ТП-277</t>
+  </si>
+  <si>
+    <t>ТП-193П</t>
   </si>
 </sst>
 </file>
@@ -1465,7 +1468,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1564,14 +1567,8 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -1580,10 +1577,19 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="26">
@@ -1614,17 +1620,7 @@
     <cellStyle name="Обычный 9" xfId="24"/>
     <cellStyle name="Обычный_Лист1" xfId="25"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1979,7 +1975,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AMI280"/>
+  <dimension ref="A1:AMI281"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.28515625" style="1" customWidth="1"/>
@@ -2005,154 +2001,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="1.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="T1" s="39" t="s">
-        <v>0</v>
-      </c>
-      <c r="U1" s="39"/>
+      <c r="T1" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="U1" s="37"/>
     </row>
     <row r="2" spans="1:22" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="T2" s="39"/>
-      <c r="U2" s="39"/>
+      <c r="T2" s="37"/>
+      <c r="U2" s="37"/>
     </row>
     <row r="3" spans="1:22" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="T3" s="39"/>
-      <c r="U3" s="39"/>
+      <c r="T3" s="37"/>
+      <c r="U3" s="37"/>
     </row>
     <row r="4" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
-      <c r="H4" s="40"/>
-      <c r="I4" s="40"/>
-      <c r="J4" s="40"/>
-      <c r="K4" s="40"/>
-      <c r="L4" s="40"/>
-      <c r="M4" s="40"/>
-      <c r="N4" s="40"/>
-      <c r="O4" s="40"/>
-      <c r="P4" s="40"/>
-      <c r="Q4" s="40"/>
-      <c r="R4" s="40"/>
-      <c r="S4" s="40"/>
-      <c r="T4" s="40"/>
-      <c r="U4" s="40"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="38"/>
+      <c r="H4" s="38"/>
+      <c r="I4" s="38"/>
+      <c r="J4" s="38"/>
+      <c r="K4" s="38"/>
+      <c r="L4" s="38"/>
+      <c r="M4" s="38"/>
+      <c r="N4" s="38"/>
+      <c r="O4" s="38"/>
+      <c r="P4" s="38"/>
+      <c r="Q4" s="38"/>
+      <c r="R4" s="38"/>
+      <c r="S4" s="38"/>
+      <c r="T4" s="38"/>
+      <c r="U4" s="38"/>
     </row>
     <row r="5" spans="1:22" ht="47.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="37" t="s">
+      <c r="C6" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="37" t="s">
+      <c r="D6" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="37" t="s">
+      <c r="E6" s="39"/>
+      <c r="F6" s="39"/>
+      <c r="G6" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="H6" s="41" t="s">
+      <c r="H6" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="I6" s="41"/>
-      <c r="J6" s="41"/>
-      <c r="K6" s="41"/>
-      <c r="L6" s="37" t="s">
+      <c r="I6" s="40"/>
+      <c r="J6" s="40"/>
+      <c r="K6" s="40"/>
+      <c r="L6" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="M6" s="37"/>
-      <c r="N6" s="37"/>
-      <c r="O6" s="37" t="s">
+      <c r="M6" s="39"/>
+      <c r="N6" s="39"/>
+      <c r="O6" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="P6" s="37" t="s">
+      <c r="P6" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="Q6" s="37" t="s">
+      <c r="Q6" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="R6" s="37"/>
-      <c r="S6" s="37"/>
-      <c r="T6" s="37"/>
-      <c r="U6" s="37" t="s">
+      <c r="R6" s="39"/>
+      <c r="S6" s="39"/>
+      <c r="T6" s="39"/>
+      <c r="U6" s="39" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="37"/>
-      <c r="B7" s="37"/>
-      <c r="C7" s="37"/>
-      <c r="D7" s="37" t="s">
+      <c r="A7" s="39"/>
+      <c r="B7" s="39"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="37" t="s">
+      <c r="F7" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37" t="s">
+      <c r="G7" s="39"/>
+      <c r="H7" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="I7" s="37" t="s">
+      <c r="I7" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="J7" s="37" t="s">
+      <c r="J7" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="K7" s="37" t="s">
+      <c r="K7" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="L7" s="37" t="s">
+      <c r="L7" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="M7" s="37" t="s">
+      <c r="M7" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="N7" s="37" t="s">
+      <c r="N7" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="O7" s="37"/>
-      <c r="P7" s="37"/>
-      <c r="Q7" s="37" t="s">
+      <c r="O7" s="39"/>
+      <c r="P7" s="39"/>
+      <c r="Q7" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="R7" s="37"/>
-      <c r="S7" s="37" t="s">
+      <c r="R7" s="39"/>
+      <c r="S7" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="T7" s="37"/>
-      <c r="U7" s="37"/>
+      <c r="T7" s="39"/>
+      <c r="U7" s="39"/>
     </row>
     <row r="8" spans="1:22" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="37"/>
-      <c r="B8" s="37"/>
-      <c r="C8" s="37"/>
-      <c r="D8" s="37"/>
-      <c r="E8" s="37"/>
-      <c r="F8" s="37"/>
-      <c r="G8" s="37"/>
-      <c r="H8" s="37"/>
-      <c r="I8" s="37"/>
-      <c r="J8" s="37"/>
-      <c r="K8" s="37"/>
-      <c r="L8" s="37"/>
-      <c r="M8" s="37"/>
-      <c r="N8" s="37"/>
-      <c r="O8" s="37"/>
-      <c r="P8" s="37"/>
+      <c r="A8" s="39"/>
+      <c r="B8" s="39"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="39"/>
+      <c r="I8" s="39"/>
+      <c r="J8" s="39"/>
+      <c r="K8" s="39"/>
+      <c r="L8" s="39"/>
+      <c r="M8" s="39"/>
+      <c r="N8" s="39"/>
+      <c r="O8" s="39"/>
+      <c r="P8" s="39"/>
       <c r="Q8" s="2" t="s">
         <v>24</v>
       </c>
@@ -2165,7 +2161,7 @@
       <c r="T8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="U8" s="37"/>
+      <c r="U8" s="39"/>
       <c r="V8" s="5"/>
     </row>
     <row r="9" spans="1:22" s="10" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -8825,14 +8821,14 @@
       <c r="K140" s="2"/>
       <c r="L140" s="11"/>
       <c r="M140" s="11">
-        <f t="shared" ref="M140:M203" si="9">L140</f>
+        <f t="shared" ref="M140:M204" si="9">L140</f>
         <v>0</v>
       </c>
       <c r="N140" s="11" t="s">
         <v>31</v>
       </c>
       <c r="O140" s="12">
-        <f t="shared" ref="O140:O203" si="10">H140-L140</f>
+        <f t="shared" ref="O140:O204" si="10">H140-L140</f>
         <v>0</v>
       </c>
       <c r="P140" s="13">
@@ -10764,7 +10760,7 @@
       </c>
       <c r="H179" s="11"/>
       <c r="I179" s="11">
-        <f t="shared" ref="I179:I210" si="12">H179-J179</f>
+        <f t="shared" ref="I179:I211" si="12">H179-J179</f>
         <v>0</v>
       </c>
       <c r="J179" s="2"/>
@@ -11286,20 +11282,20 @@
       <c r="V189" s="5"/>
     </row>
     <row r="190" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A190" s="2">
+      <c r="A190" s="36">
         <v>181</v>
       </c>
       <c r="B190" s="11" t="s">
-        <v>281</v>
-      </c>
-      <c r="C190" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="C190" s="36" t="s">
         <v>73</v>
       </c>
-      <c r="D190" s="2"/>
-      <c r="E190" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F190" s="2" t="s">
+      <c r="D190" s="36"/>
+      <c r="E190" s="36" t="s">
+        <v>348</v>
+      </c>
+      <c r="F190" s="36" t="s">
         <v>41</v>
       </c>
       <c r="G190" s="11">
@@ -11310,8 +11306,8 @@
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J190" s="2"/>
-      <c r="K190" s="2"/>
+      <c r="J190" s="36"/>
+      <c r="K190" s="36"/>
       <c r="L190" s="11"/>
       <c r="M190" s="11">
         <f t="shared" si="9"/>
@@ -11320,7 +11316,7 @@
       <c r="N190" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="O190" s="12">
+      <c r="O190" s="21">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
@@ -11335,11 +11331,11 @@
       <c r="V190" s="5"/>
     </row>
     <row r="191" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A191" s="2">
+      <c r="A191" s="36">
         <v>182</v>
       </c>
       <c r="B191" s="11" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C191" s="2" t="s">
         <v>73</v>
@@ -11384,11 +11380,11 @@
       <c r="V191" s="5"/>
     </row>
     <row r="192" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A192" s="2">
+      <c r="A192" s="36">
         <v>183</v>
       </c>
       <c r="B192" s="11" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C192" s="2" t="s">
         <v>73</v>
@@ -11433,26 +11429,24 @@
       <c r="V192" s="5"/>
     </row>
     <row r="193" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A193" s="2">
+      <c r="A193" s="36">
         <v>184</v>
       </c>
       <c r="B193" s="11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D193" s="2" t="s">
-        <v>28</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="D193" s="2"/>
       <c r="E193" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F193" s="2" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="G193" s="11">
-        <v>164</v>
+        <v>1</v>
       </c>
       <c r="H193" s="11"/>
       <c r="I193" s="11">
@@ -11467,7 +11461,7 @@
         <v>0</v>
       </c>
       <c r="N193" s="11" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="O193" s="12">
         <f t="shared" si="10"/>
@@ -11484,14 +11478,14 @@
       <c r="V193" s="5"/>
     </row>
     <row r="194" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A194" s="2">
+      <c r="A194" s="36">
         <v>185</v>
       </c>
       <c r="B194" s="11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="D194" s="2" t="s">
         <v>28</v>
@@ -11500,10 +11494,10 @@
         <v>29</v>
       </c>
       <c r="F194" s="2" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="G194" s="11">
-        <v>1</v>
+        <v>164</v>
       </c>
       <c r="H194" s="11"/>
       <c r="I194" s="11">
@@ -11518,7 +11512,7 @@
         <v>0</v>
       </c>
       <c r="N194" s="11" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="O194" s="12">
         <f t="shared" si="10"/>
@@ -11535,26 +11529,26 @@
       <c r="V194" s="5"/>
     </row>
     <row r="195" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A195" s="2">
+      <c r="A195" s="36">
         <v>186</v>
       </c>
       <c r="B195" s="11" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>27</v>
+        <v>73</v>
       </c>
       <c r="D195" s="2" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="E195" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F195" s="2" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="G195" s="11">
-        <v>76</v>
+        <v>1</v>
       </c>
       <c r="H195" s="11"/>
       <c r="I195" s="11">
@@ -11569,7 +11563,7 @@
         <v>0</v>
       </c>
       <c r="N195" s="11" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="O195" s="12">
         <f t="shared" si="10"/>
@@ -11586,11 +11580,11 @@
       <c r="V195" s="5"/>
     </row>
     <row r="196" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A196" s="2">
+      <c r="A196" s="36">
         <v>187</v>
       </c>
       <c r="B196" s="11" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C196" s="2" t="s">
         <v>27</v>
@@ -11605,7 +11599,7 @@
         <v>30</v>
       </c>
       <c r="G196" s="11">
-        <v>114</v>
+        <v>76</v>
       </c>
       <c r="H196" s="11"/>
       <c r="I196" s="11">
@@ -11620,7 +11614,7 @@
         <v>0</v>
       </c>
       <c r="N196" s="11" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="O196" s="12">
         <f t="shared" si="10"/>
@@ -11637,26 +11631,26 @@
       <c r="V196" s="5"/>
     </row>
     <row r="197" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A197" s="2">
+      <c r="A197" s="36">
         <v>188</v>
       </c>
       <c r="B197" s="11" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C197" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D197" s="2" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="E197" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F197" s="2" t="s">
-        <v>289</v>
+        <v>30</v>
       </c>
       <c r="G197" s="11">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="H197" s="11"/>
       <c r="I197" s="11">
@@ -11671,7 +11665,7 @@
         <v>0</v>
       </c>
       <c r="N197" s="11" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="O197" s="12">
         <f t="shared" si="10"/>
@@ -11688,24 +11682,26 @@
       <c r="V197" s="5"/>
     </row>
     <row r="198" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A198" s="2">
+      <c r="A198" s="36">
         <v>189</v>
       </c>
       <c r="B198" s="11" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D198" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="D198" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="E198" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F198" s="2" t="s">
-        <v>41</v>
+        <v>289</v>
       </c>
       <c r="G198" s="11">
-        <v>1</v>
+        <v>91</v>
       </c>
       <c r="H198" s="11"/>
       <c r="I198" s="11">
@@ -11720,7 +11716,7 @@
         <v>0</v>
       </c>
       <c r="N198" s="11" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="O198" s="12">
         <f t="shared" si="10"/>
@@ -11737,26 +11733,24 @@
       <c r="V198" s="5"/>
     </row>
     <row r="199" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A199" s="2">
+      <c r="A199" s="36">
         <v>190</v>
       </c>
       <c r="B199" s="11" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D199" s="2" t="s">
-        <v>54</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="D199" s="2"/>
       <c r="E199" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F199" s="2" t="s">
-        <v>150</v>
+        <v>41</v>
       </c>
       <c r="G199" s="11">
-        <v>107</v>
+        <v>1</v>
       </c>
       <c r="H199" s="11"/>
       <c r="I199" s="11">
@@ -11771,7 +11765,7 @@
         <v>0</v>
       </c>
       <c r="N199" s="11" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="O199" s="12">
         <f t="shared" si="10"/>
@@ -11788,26 +11782,26 @@
       <c r="V199" s="5"/>
     </row>
     <row r="200" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A200" s="2">
+      <c r="A200" s="36">
         <v>191</v>
       </c>
       <c r="B200" s="11" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C200" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D200" s="2" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="E200" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F200" s="2" t="s">
-        <v>34</v>
+        <v>150</v>
       </c>
       <c r="G200" s="11">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="H200" s="11"/>
       <c r="I200" s="11">
@@ -11821,8 +11815,8 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="N200" s="15" t="s">
-        <v>293</v>
+      <c r="N200" s="11" t="s">
+        <v>31</v>
       </c>
       <c r="O200" s="12">
         <f t="shared" si="10"/>
@@ -11839,24 +11833,26 @@
       <c r="V200" s="5"/>
     </row>
     <row r="201" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A201" s="2">
+      <c r="A201" s="36">
         <v>192</v>
       </c>
       <c r="B201" s="11" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D201" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="D201" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="E201" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F201" s="2" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="G201" s="11">
-        <v>1</v>
+        <v>103</v>
       </c>
       <c r="H201" s="11"/>
       <c r="I201" s="11">
@@ -11870,8 +11866,8 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="N201" s="11" t="s">
-        <v>50</v>
+      <c r="N201" s="15" t="s">
+        <v>293</v>
       </c>
       <c r="O201" s="12">
         <f t="shared" si="10"/>
@@ -11888,11 +11884,11 @@
       <c r="V201" s="5"/>
     </row>
     <row r="202" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A202" s="2">
+      <c r="A202" s="36">
         <v>193</v>
       </c>
       <c r="B202" s="11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C202" s="2" t="s">
         <v>73</v>
@@ -11937,26 +11933,24 @@
       <c r="V202" s="5"/>
     </row>
     <row r="203" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A203" s="2">
+      <c r="A203" s="36">
         <v>194</v>
       </c>
       <c r="B203" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D203" s="2" t="s">
-        <v>28</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="D203" s="2"/>
       <c r="E203" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F203" s="2" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="G203" s="11">
-        <v>164</v>
+        <v>1</v>
       </c>
       <c r="H203" s="11"/>
       <c r="I203" s="11">
@@ -11970,8 +11964,8 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="N203" s="15" t="s">
-        <v>117</v>
+      <c r="N203" s="11" t="s">
+        <v>50</v>
       </c>
       <c r="O203" s="12">
         <f t="shared" si="10"/>
@@ -11988,24 +11982,26 @@
       <c r="V203" s="5"/>
     </row>
     <row r="204" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A204" s="2">
+      <c r="A204" s="36">
         <v>195</v>
       </c>
       <c r="B204" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D204" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="D204" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="E204" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F204" s="2" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="G204" s="11">
-        <v>1</v>
+        <v>164</v>
       </c>
       <c r="H204" s="11"/>
       <c r="I204" s="11">
@@ -12016,14 +12012,14 @@
       <c r="K204" s="2"/>
       <c r="L204" s="11"/>
       <c r="M204" s="11">
-        <f t="shared" ref="M204:M268" si="13">L204</f>
-        <v>0</v>
-      </c>
-      <c r="N204" s="11" t="s">
-        <v>50</v>
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="N204" s="15" t="s">
+        <v>117</v>
       </c>
       <c r="O204" s="12">
-        <f t="shared" ref="O204:O272" si="14">H204-L204</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="P204" s="13">
@@ -12037,11 +12033,11 @@
       <c r="V204" s="5"/>
     </row>
     <row r="205" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A205" s="2">
+      <c r="A205" s="36">
         <v>196</v>
       </c>
       <c r="B205" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C205" s="2" t="s">
         <v>73</v>
@@ -12065,14 +12061,14 @@
       <c r="K205" s="2"/>
       <c r="L205" s="11"/>
       <c r="M205" s="11">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="M205:M269" si="13">L205</f>
         <v>0</v>
       </c>
       <c r="N205" s="11" t="s">
         <v>50</v>
       </c>
       <c r="O205" s="12">
-        <f t="shared" si="14"/>
+        <f t="shared" ref="O205:O273" si="14">H205-L205</f>
         <v>0</v>
       </c>
       <c r="P205" s="13">
@@ -12086,11 +12082,11 @@
       <c r="V205" s="5"/>
     </row>
     <row r="206" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A206" s="2">
+      <c r="A206" s="36">
         <v>197</v>
       </c>
       <c r="B206" s="11" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C206" s="2" t="s">
         <v>73</v>
@@ -12135,26 +12131,24 @@
       <c r="V206" s="5"/>
     </row>
     <row r="207" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A207" s="2">
+      <c r="A207" s="36">
         <v>198</v>
       </c>
       <c r="B207" s="11" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D207" s="2" t="s">
-        <v>28</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="D207" s="2"/>
       <c r="E207" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F207" s="2" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="G207" s="11">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="H207" s="11"/>
       <c r="I207" s="11">
@@ -12168,8 +12162,8 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="N207" s="15" t="s">
-        <v>168</v>
+      <c r="N207" s="11" t="s">
+        <v>50</v>
       </c>
       <c r="O207" s="12">
         <f t="shared" si="14"/>
@@ -12186,24 +12180,26 @@
       <c r="V207" s="5"/>
     </row>
     <row r="208" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A208" s="2">
+      <c r="A208" s="36">
         <v>199</v>
       </c>
       <c r="B208" s="11" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D208" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="D208" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="E208" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F208" s="2" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="G208" s="11">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="H208" s="11"/>
       <c r="I208" s="11">
@@ -12217,8 +12213,8 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="N208" s="11" t="s">
-        <v>50</v>
+      <c r="N208" s="15" t="s">
+        <v>168</v>
       </c>
       <c r="O208" s="12">
         <f t="shared" si="14"/>
@@ -12235,11 +12231,11 @@
       <c r="V208" s="5"/>
     </row>
     <row r="209" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A209" s="2">
+      <c r="A209" s="36">
         <v>200</v>
       </c>
       <c r="B209" s="11" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C209" s="2" t="s">
         <v>73</v>
@@ -12284,11 +12280,11 @@
       <c r="V209" s="5"/>
     </row>
     <row r="210" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A210" s="2">
+      <c r="A210" s="36">
         <v>201</v>
       </c>
       <c r="B210" s="11" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C210" s="2" t="s">
         <v>73</v>
@@ -12333,11 +12329,11 @@
       <c r="V210" s="5"/>
     </row>
     <row r="211" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A211" s="2">
+      <c r="A211" s="36">
         <v>202</v>
       </c>
       <c r="B211" s="11" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C211" s="2" t="s">
         <v>73</v>
@@ -12354,7 +12350,7 @@
       </c>
       <c r="H211" s="11"/>
       <c r="I211" s="11">
-        <f t="shared" ref="I211:I242" si="15">H211-J211</f>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="J211" s="2"/>
@@ -12382,11 +12378,11 @@
       <c r="V211" s="5"/>
     </row>
     <row r="212" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A212" s="2">
+      <c r="A212" s="36">
         <v>203</v>
       </c>
       <c r="B212" s="11" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C212" s="2" t="s">
         <v>73</v>
@@ -12399,11 +12395,11 @@
         <v>41</v>
       </c>
       <c r="G212" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H212" s="11"/>
       <c r="I212" s="11">
-        <f t="shared" si="15"/>
+        <f t="shared" ref="I212:I243" si="15">H212-J212</f>
         <v>0</v>
       </c>
       <c r="J212" s="2"/>
@@ -12431,26 +12427,24 @@
       <c r="V212" s="5"/>
     </row>
     <row r="213" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A213" s="2">
+      <c r="A213" s="36">
         <v>204</v>
       </c>
       <c r="B213" s="11" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C213" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D213" s="2" t="s">
-        <v>28</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="D213" s="2"/>
       <c r="E213" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F213" s="2" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="G213" s="11">
-        <v>86</v>
+        <v>2</v>
       </c>
       <c r="H213" s="11"/>
       <c r="I213" s="11">
@@ -12464,8 +12458,8 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="N213" s="15" t="s">
-        <v>117</v>
+      <c r="N213" s="11" t="s">
+        <v>50</v>
       </c>
       <c r="O213" s="12">
         <f t="shared" si="14"/>
@@ -12482,17 +12476,17 @@
       <c r="V213" s="5"/>
     </row>
     <row r="214" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A214" s="2">
+      <c r="A214" s="36">
         <v>205</v>
       </c>
       <c r="B214" s="11" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C214" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D214" s="2" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="E214" s="2" t="s">
         <v>29</v>
@@ -12501,7 +12495,7 @@
         <v>34</v>
       </c>
       <c r="G214" s="11">
-        <v>119</v>
+        <v>86</v>
       </c>
       <c r="H214" s="11"/>
       <c r="I214" s="11">
@@ -12516,7 +12510,7 @@
         <v>0</v>
       </c>
       <c r="N214" s="15" t="s">
-        <v>262</v>
+        <v>117</v>
       </c>
       <c r="O214" s="12">
         <f t="shared" si="14"/>
@@ -12533,24 +12527,26 @@
       <c r="V214" s="5"/>
     </row>
     <row r="215" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A215" s="2">
+      <c r="A215" s="36">
         <v>206</v>
       </c>
       <c r="B215" s="11" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C215" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D215" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="D215" s="2" t="s">
+        <v>54</v>
+      </c>
       <c r="E215" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F215" s="2" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="G215" s="11">
-        <v>1</v>
+        <v>119</v>
       </c>
       <c r="H215" s="11"/>
       <c r="I215" s="11">
@@ -12564,8 +12560,8 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="N215" s="11" t="s">
-        <v>50</v>
+      <c r="N215" s="15" t="s">
+        <v>262</v>
       </c>
       <c r="O215" s="12">
         <f t="shared" si="14"/>
@@ -12582,11 +12578,11 @@
       <c r="V215" s="5"/>
     </row>
     <row r="216" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A216" s="2">
+      <c r="A216" s="36">
         <v>207</v>
       </c>
       <c r="B216" s="11" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C216" s="2" t="s">
         <v>73</v>
@@ -12631,26 +12627,24 @@
       <c r="V216" s="5"/>
     </row>
     <row r="217" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A217" s="2">
+      <c r="A217" s="36">
         <v>208</v>
       </c>
       <c r="B217" s="11" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C217" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D217" s="2" t="s">
-        <v>138</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="D217" s="2"/>
       <c r="E217" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F217" s="2" t="s">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="G217" s="11">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="H217" s="11"/>
       <c r="I217" s="11">
@@ -12664,14 +12658,14 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="N217" s="16" t="s">
-        <v>311</v>
+      <c r="N217" s="11" t="s">
+        <v>50</v>
       </c>
       <c r="O217" s="12">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P217" s="11">
+      <c r="P217" s="13">
         <v>0</v>
       </c>
       <c r="Q217" s="14"/>
@@ -12682,24 +12676,26 @@
       <c r="V217" s="5"/>
     </row>
     <row r="218" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A218" s="2">
+      <c r="A218" s="36">
         <v>209</v>
       </c>
       <c r="B218" s="11" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C218" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D218" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="D218" s="2" t="s">
+        <v>138</v>
+      </c>
       <c r="E218" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F218" s="2" t="s">
-        <v>41</v>
+        <v>100</v>
       </c>
       <c r="G218" s="11">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="H218" s="11"/>
       <c r="I218" s="11">
@@ -12713,14 +12709,14 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="N218" s="11" t="s">
-        <v>50</v>
+      <c r="N218" s="16" t="s">
+        <v>311</v>
       </c>
       <c r="O218" s="12">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P218" s="13">
+      <c r="P218" s="11">
         <v>0</v>
       </c>
       <c r="Q218" s="14"/>
@@ -12731,11 +12727,11 @@
       <c r="V218" s="5"/>
     </row>
     <row r="219" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A219" s="2">
+      <c r="A219" s="36">
         <v>210</v>
       </c>
       <c r="B219" s="11" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C219" s="2" t="s">
         <v>73</v>
@@ -12780,11 +12776,11 @@
       <c r="V219" s="5"/>
     </row>
     <row r="220" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A220" s="2">
+      <c r="A220" s="36">
         <v>211</v>
       </c>
       <c r="B220" s="11" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C220" s="2" t="s">
         <v>73</v>
@@ -12829,11 +12825,11 @@
       <c r="V220" s="5"/>
     </row>
     <row r="221" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A221" s="2">
+      <c r="A221" s="36">
         <v>212</v>
       </c>
       <c r="B221" s="11" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C221" s="2" t="s">
         <v>73</v>
@@ -12878,26 +12874,24 @@
       <c r="V221" s="5"/>
     </row>
     <row r="222" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A222" s="2">
+      <c r="A222" s="36">
         <v>213</v>
       </c>
       <c r="B222" s="11" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C222" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D222" s="2" t="s">
-        <v>317</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="D222" s="2"/>
       <c r="E222" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F222" s="2" t="s">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="G222" s="11">
-        <v>64</v>
+        <v>1</v>
       </c>
       <c r="H222" s="11"/>
       <c r="I222" s="11">
@@ -12912,13 +12906,13 @@
         <v>0</v>
       </c>
       <c r="N222" s="11" t="s">
-        <v>318</v>
+        <v>50</v>
       </c>
       <c r="O222" s="12">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P222" s="11">
+      <c r="P222" s="13">
         <v>0</v>
       </c>
       <c r="Q222" s="14"/>
@@ -12929,17 +12923,17 @@
       <c r="V222" s="5"/>
     </row>
     <row r="223" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A223" s="2">
+      <c r="A223" s="36">
         <v>214</v>
       </c>
       <c r="B223" s="11" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="C223" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D223" s="2" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="E223" s="2" t="s">
         <v>29</v>
@@ -12948,7 +12942,7 @@
         <v>100</v>
       </c>
       <c r="G223" s="11">
-        <v>94</v>
+        <v>64</v>
       </c>
       <c r="H223" s="11"/>
       <c r="I223" s="11">
@@ -12963,7 +12957,7 @@
         <v>0</v>
       </c>
       <c r="N223" s="11" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="O223" s="12">
         <f t="shared" si="14"/>
@@ -12980,26 +12974,26 @@
       <c r="V223" s="5"/>
     </row>
     <row r="224" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A224" s="2">
+      <c r="A224" s="36">
         <v>215</v>
       </c>
       <c r="B224" s="11" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="C224" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D224" s="2" t="s">
-        <v>255</v>
+        <v>320</v>
       </c>
       <c r="E224" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F224" s="2" t="s">
-        <v>34</v>
+        <v>100</v>
       </c>
       <c r="G224" s="11">
-        <v>3</v>
+        <v>94</v>
       </c>
       <c r="H224" s="11"/>
       <c r="I224" s="11">
@@ -13013,12 +13007,14 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="N224" s="11"/>
+      <c r="N224" s="11" t="s">
+        <v>321</v>
+      </c>
       <c r="O224" s="12">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P224" s="13">
+      <c r="P224" s="11">
         <v>0</v>
       </c>
       <c r="Q224" s="14"/>
@@ -13029,24 +13025,26 @@
       <c r="V224" s="5"/>
     </row>
     <row r="225" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A225" s="2">
+      <c r="A225" s="36">
         <v>216</v>
       </c>
       <c r="B225" s="11" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C225" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D225" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="D225" s="2" t="s">
+        <v>255</v>
+      </c>
       <c r="E225" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F225" s="2" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="G225" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H225" s="11"/>
       <c r="I225" s="11">
@@ -13060,9 +13058,7 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="N225" s="11" t="s">
-        <v>50</v>
-      </c>
+      <c r="N225" s="11"/>
       <c r="O225" s="12">
         <f t="shared" si="14"/>
         <v>0</v>
@@ -13078,26 +13074,24 @@
       <c r="V225" s="5"/>
     </row>
     <row r="226" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A226" s="2">
+      <c r="A226" s="36">
         <v>217</v>
       </c>
       <c r="B226" s="11" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C226" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D226" s="2" t="s">
-        <v>37</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="D226" s="2"/>
       <c r="E226" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F226" s="2" t="s">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="G226" s="11">
-        <v>114</v>
+        <v>1</v>
       </c>
       <c r="H226" s="11"/>
       <c r="I226" s="11">
@@ -13112,7 +13106,7 @@
         <v>0</v>
       </c>
       <c r="N226" s="11" t="s">
-        <v>325</v>
+        <v>50</v>
       </c>
       <c r="O226" s="12">
         <f t="shared" si="14"/>
@@ -13129,11 +13123,11 @@
       <c r="V226" s="5"/>
     </row>
     <row r="227" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A227" s="2">
+      <c r="A227" s="36">
         <v>218</v>
       </c>
       <c r="B227" s="11" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C227" s="2" t="s">
         <v>27</v>
@@ -13148,7 +13142,7 @@
         <v>100</v>
       </c>
       <c r="G227" s="11">
-        <v>41</v>
+        <v>114</v>
       </c>
       <c r="H227" s="11"/>
       <c r="I227" s="11">
@@ -13163,13 +13157,13 @@
         <v>0</v>
       </c>
       <c r="N227" s="11" t="s">
-        <v>153</v>
+        <v>325</v>
       </c>
       <c r="O227" s="12">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P227" s="11">
+      <c r="P227" s="13">
         <v>0</v>
       </c>
       <c r="Q227" s="14"/>
@@ -13180,11 +13174,11 @@
       <c r="V227" s="5"/>
     </row>
     <row r="228" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A228" s="2">
+      <c r="A228" s="36">
         <v>219</v>
       </c>
       <c r="B228" s="11" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C228" s="2" t="s">
         <v>27</v>
@@ -13199,7 +13193,7 @@
         <v>100</v>
       </c>
       <c r="G228" s="11">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="H228" s="11"/>
       <c r="I228" s="11">
@@ -13214,7 +13208,7 @@
         <v>0</v>
       </c>
       <c r="N228" s="11" t="s">
-        <v>31</v>
+        <v>153</v>
       </c>
       <c r="O228" s="12">
         <f t="shared" si="14"/>
@@ -13231,11 +13225,11 @@
       <c r="V228" s="5"/>
     </row>
     <row r="229" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A229" s="2">
+      <c r="A229" s="36">
         <v>220</v>
       </c>
       <c r="B229" s="11" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C229" s="2" t="s">
         <v>27</v>
@@ -13247,10 +13241,10 @@
         <v>29</v>
       </c>
       <c r="F229" s="2" t="s">
-        <v>329</v>
+        <v>100</v>
       </c>
       <c r="G229" s="11">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="H229" s="11"/>
       <c r="I229" s="11">
@@ -13265,13 +13259,13 @@
         <v>0</v>
       </c>
       <c r="N229" s="11" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="O229" s="12">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P229" s="13">
+      <c r="P229" s="11">
         <v>0</v>
       </c>
       <c r="Q229" s="14"/>
@@ -13282,26 +13276,26 @@
       <c r="V229" s="5"/>
     </row>
     <row r="230" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A230" s="2">
+      <c r="A230" s="36">
         <v>221</v>
       </c>
       <c r="B230" s="11" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C230" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D230" s="2" t="s">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="E230" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F230" s="2" t="s">
-        <v>30</v>
+        <v>329</v>
       </c>
       <c r="G230" s="11">
-        <v>163</v>
+        <v>31</v>
       </c>
       <c r="H230" s="11"/>
       <c r="I230" s="11">
@@ -13316,7 +13310,7 @@
         <v>0</v>
       </c>
       <c r="N230" s="11" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="O230" s="12">
         <f t="shared" si="14"/>
@@ -13329,28 +13323,30 @@
       <c r="R230" s="14"/>
       <c r="S230" s="14"/>
       <c r="T230" s="14"/>
-      <c r="U230" s="2"/>
+      <c r="U230" s="14"/>
       <c r="V230" s="5"/>
     </row>
     <row r="231" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A231" s="2">
+      <c r="A231" s="36">
         <v>222</v>
       </c>
       <c r="B231" s="11" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C231" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D231" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="D231" s="2" t="s">
+        <v>67</v>
+      </c>
       <c r="E231" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F231" s="2" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="G231" s="11">
-        <v>1</v>
+        <v>163</v>
       </c>
       <c r="H231" s="11"/>
       <c r="I231" s="11">
@@ -13365,7 +13361,7 @@
         <v>0</v>
       </c>
       <c r="N231" s="11" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="O231" s="12">
         <f t="shared" si="14"/>
@@ -13382,11 +13378,11 @@
       <c r="V231" s="5"/>
     </row>
     <row r="232" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A232" s="2">
+      <c r="A232" s="36">
         <v>223</v>
       </c>
       <c r="B232" s="11" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C232" s="2" t="s">
         <v>73</v>
@@ -13431,26 +13427,24 @@
       <c r="V232" s="5"/>
     </row>
     <row r="233" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A233" s="2">
+      <c r="A233" s="36">
         <v>224</v>
       </c>
       <c r="B233" s="11" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C233" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D233" s="2" t="s">
-        <v>255</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="D233" s="2"/>
       <c r="E233" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F233" s="2" t="s">
-        <v>150</v>
+        <v>41</v>
       </c>
       <c r="G233" s="11">
-        <v>64</v>
+        <v>1</v>
       </c>
       <c r="H233" s="11"/>
       <c r="I233" s="11">
@@ -13465,7 +13459,7 @@
         <v>0</v>
       </c>
       <c r="N233" s="11" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="O233" s="12">
         <f t="shared" si="14"/>
@@ -13482,24 +13476,26 @@
       <c r="V233" s="5"/>
     </row>
     <row r="234" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A234" s="2">
+      <c r="A234" s="36">
         <v>225</v>
       </c>
       <c r="B234" s="11" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C234" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D234" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="D234" s="2" t="s">
+        <v>255</v>
+      </c>
       <c r="E234" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F234" s="2" t="s">
-        <v>41</v>
+        <v>150</v>
       </c>
       <c r="G234" s="11">
-        <v>1</v>
+        <v>64</v>
       </c>
       <c r="H234" s="11"/>
       <c r="I234" s="11">
@@ -13514,7 +13510,7 @@
         <v>0</v>
       </c>
       <c r="N234" s="11" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="O234" s="12">
         <f t="shared" si="14"/>
@@ -13531,26 +13527,24 @@
       <c r="V234" s="5"/>
     </row>
     <row r="235" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A235" s="2">
+      <c r="A235" s="36">
         <v>226</v>
       </c>
       <c r="B235" s="11" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C235" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D235" s="2" t="s">
-        <v>152</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="D235" s="2"/>
       <c r="E235" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F235" s="2" t="s">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="G235" s="11">
-        <v>59</v>
+        <v>1</v>
       </c>
       <c r="H235" s="11"/>
       <c r="I235" s="11">
@@ -13565,7 +13559,7 @@
         <v>0</v>
       </c>
       <c r="N235" s="11" t="s">
-        <v>336</v>
+        <v>50</v>
       </c>
       <c r="O235" s="12">
         <f t="shared" si="14"/>
@@ -13582,11 +13576,11 @@
       <c r="V235" s="5"/>
     </row>
     <row r="236" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A236" s="2">
+      <c r="A236" s="36">
         <v>227</v>
       </c>
       <c r="B236" s="11" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C236" s="2" t="s">
         <v>27</v>
@@ -13601,7 +13595,7 @@
         <v>100</v>
       </c>
       <c r="G236" s="11">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="H236" s="11"/>
       <c r="I236" s="11">
@@ -13616,28 +13610,28 @@
         <v>0</v>
       </c>
       <c r="N236" s="11" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="O236" s="12">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P236" s="11">
+      <c r="P236" s="13">
         <v>0</v>
       </c>
       <c r="Q236" s="14"/>
       <c r="R236" s="14"/>
       <c r="S236" s="14"/>
       <c r="T236" s="14"/>
-      <c r="U236" s="14"/>
+      <c r="U236" s="2"/>
       <c r="V236" s="5"/>
     </row>
     <row r="237" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A237" s="2">
+      <c r="A237" s="36">
         <v>228</v>
       </c>
       <c r="B237" s="11" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C237" s="2" t="s">
         <v>27</v>
@@ -13652,7 +13646,7 @@
         <v>100</v>
       </c>
       <c r="G237" s="11">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="H237" s="11"/>
       <c r="I237" s="11">
@@ -13667,7 +13661,7 @@
         <v>0</v>
       </c>
       <c r="N237" s="11" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="O237" s="12">
         <f t="shared" si="14"/>
@@ -13684,11 +13678,11 @@
       <c r="V237" s="5"/>
     </row>
     <row r="238" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A238" s="2">
+      <c r="A238" s="36">
         <v>229</v>
       </c>
       <c r="B238" s="11" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C238" s="2" t="s">
         <v>27</v>
@@ -13703,7 +13697,7 @@
         <v>100</v>
       </c>
       <c r="G238" s="11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H238" s="11"/>
       <c r="I238" s="11">
@@ -13718,7 +13712,7 @@
         <v>0</v>
       </c>
       <c r="N238" s="11" t="s">
-        <v>31</v>
+        <v>340</v>
       </c>
       <c r="O238" s="12">
         <f t="shared" si="14"/>
@@ -13735,26 +13729,26 @@
       <c r="V238" s="5"/>
     </row>
     <row r="239" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A239" s="2">
+      <c r="A239" s="36">
         <v>230</v>
       </c>
       <c r="B239" s="11" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C239" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D239" s="2" t="s">
-        <v>79</v>
+        <v>152</v>
       </c>
       <c r="E239" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F239" s="2" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="G239" s="11">
-        <v>135</v>
+        <v>3</v>
       </c>
       <c r="H239" s="11"/>
       <c r="I239" s="11">
@@ -13786,11 +13780,11 @@
       <c r="V239" s="5"/>
     </row>
     <row r="240" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A240" s="2">
+      <c r="A240" s="36">
         <v>231</v>
       </c>
       <c r="B240" s="11" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C240" s="2" t="s">
         <v>27</v>
@@ -13802,10 +13796,10 @@
         <v>29</v>
       </c>
       <c r="F240" s="2" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="G240" s="11">
-        <v>23</v>
+        <v>135</v>
       </c>
       <c r="H240" s="11"/>
       <c r="I240" s="11">
@@ -13837,11 +13831,11 @@
       <c r="V240" s="5"/>
     </row>
     <row r="241" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A241" s="2">
+      <c r="A241" s="36">
         <v>232</v>
       </c>
       <c r="B241" s="11" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C241" s="2" t="s">
         <v>27</v>
@@ -13856,7 +13850,7 @@
         <v>100</v>
       </c>
       <c r="G241" s="11">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="H241" s="11"/>
       <c r="I241" s="11">
@@ -13870,14 +13864,14 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="N241" s="15" t="s">
-        <v>345</v>
+      <c r="N241" s="11" t="s">
+        <v>31</v>
       </c>
       <c r="O241" s="12">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P241" s="13">
+      <c r="P241" s="11">
         <v>0</v>
       </c>
       <c r="Q241" s="14"/>
@@ -13888,11 +13882,11 @@
       <c r="V241" s="5"/>
     </row>
     <row r="242" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A242" s="2">
+      <c r="A242" s="36">
         <v>233</v>
       </c>
       <c r="B242" s="11" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C242" s="2" t="s">
         <v>27</v>
@@ -13907,7 +13901,7 @@
         <v>100</v>
       </c>
       <c r="G242" s="11">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H242" s="11"/>
       <c r="I242" s="11">
@@ -13921,8 +13915,8 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="N242" s="11" t="s">
-        <v>31</v>
+      <c r="N242" s="15" t="s">
+        <v>345</v>
       </c>
       <c r="O242" s="12">
         <f t="shared" si="14"/>
@@ -13939,28 +13933,30 @@
       <c r="V242" s="5"/>
     </row>
     <row r="243" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A243" s="2">
+      <c r="A243" s="36">
         <v>234</v>
       </c>
       <c r="B243" s="11" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C243" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D243" s="2"/>
+      <c r="D243" s="2" t="s">
+        <v>79</v>
+      </c>
       <c r="E243" s="2" t="s">
-        <v>348</v>
+        <v>29</v>
       </c>
       <c r="F243" s="2" t="s">
-        <v>317</v>
+        <v>100</v>
       </c>
       <c r="G243" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H243" s="11"/>
       <c r="I243" s="11">
-        <f t="shared" ref="I243:I262" si="16">H243-J243</f>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="J243" s="2"/>
@@ -13971,7 +13967,7 @@
         <v>0</v>
       </c>
       <c r="N243" s="11" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="O243" s="12">
         <f t="shared" si="14"/>
@@ -13988,28 +13984,28 @@
       <c r="V243" s="5"/>
     </row>
     <row r="244" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A244" s="2">
+      <c r="A244" s="36">
         <v>235</v>
       </c>
       <c r="B244" s="11" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C244" s="2" t="s">
-        <v>124</v>
+        <v>27</v>
       </c>
       <c r="D244" s="2"/>
       <c r="E244" s="2" t="s">
-        <v>29</v>
+        <v>348</v>
       </c>
       <c r="F244" s="2" t="s">
-        <v>41</v>
+        <v>317</v>
       </c>
       <c r="G244" s="11">
         <v>1</v>
       </c>
       <c r="H244" s="11"/>
       <c r="I244" s="11">
-        <f t="shared" si="16"/>
+        <f t="shared" ref="I244:I263" si="16">H244-J244</f>
         <v>0</v>
       </c>
       <c r="J244" s="2"/>
@@ -14037,26 +14033,24 @@
       <c r="V244" s="5"/>
     </row>
     <row r="245" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A245" s="2">
+      <c r="A245" s="36">
         <v>236</v>
       </c>
       <c r="B245" s="11" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C245" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D245" s="2" t="s">
-        <v>79</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="D245" s="2"/>
       <c r="E245" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F245" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G245" s="11">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H245" s="11"/>
       <c r="I245" s="11">
@@ -14071,7 +14065,7 @@
         <v>0</v>
       </c>
       <c r="N245" s="11" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="O245" s="12">
         <f t="shared" si="14"/>
@@ -14088,11 +14082,11 @@
       <c r="V245" s="5"/>
     </row>
     <row r="246" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A246" s="2">
+      <c r="A246" s="36">
         <v>237</v>
       </c>
       <c r="B246" s="11" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C246" s="2" t="s">
         <v>27</v>
@@ -14104,7 +14098,7 @@
         <v>29</v>
       </c>
       <c r="F246" s="2" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="G246" s="11">
         <v>4</v>
@@ -14139,11 +14133,11 @@
       <c r="V246" s="5"/>
     </row>
     <row r="247" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A247" s="2">
+      <c r="A247" s="36">
         <v>238</v>
       </c>
       <c r="B247" s="11" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C247" s="2" t="s">
         <v>27</v>
@@ -14158,7 +14152,7 @@
         <v>100</v>
       </c>
       <c r="G247" s="11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H247" s="11"/>
       <c r="I247" s="11">
@@ -14179,7 +14173,9 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P247" s="13"/>
+      <c r="P247" s="13">
+        <v>0</v>
+      </c>
       <c r="Q247" s="14"/>
       <c r="R247" s="14"/>
       <c r="S247" s="14"/>
@@ -14188,26 +14184,26 @@
       <c r="V247" s="5"/>
     </row>
     <row r="248" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A248" s="2">
+      <c r="A248" s="36">
         <v>239</v>
       </c>
       <c r="B248" s="11" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C248" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D248" s="2" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="E248" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F248" s="2" t="s">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="G248" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H248" s="11"/>
       <c r="I248" s="11">
@@ -14228,9 +14224,7 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P248" s="13">
-        <v>0</v>
-      </c>
+      <c r="P248" s="13"/>
       <c r="Q248" s="14"/>
       <c r="R248" s="14"/>
       <c r="S248" s="14"/>
@@ -14239,11 +14233,11 @@
       <c r="V248" s="5"/>
     </row>
     <row r="249" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A249" s="2">
+      <c r="A249" s="36">
         <v>240</v>
       </c>
       <c r="B249" s="11" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C249" s="2" t="s">
         <v>27</v>
@@ -14258,7 +14252,7 @@
         <v>30</v>
       </c>
       <c r="G249" s="11">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H249" s="11"/>
       <c r="I249" s="11">
@@ -14290,11 +14284,11 @@
       <c r="V249" s="5"/>
     </row>
     <row r="250" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A250" s="2">
+      <c r="A250" s="36">
         <v>241</v>
       </c>
       <c r="B250" s="11" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C250" s="2" t="s">
         <v>27</v>
@@ -14306,10 +14300,10 @@
         <v>29</v>
       </c>
       <c r="F250" s="2" t="s">
-        <v>150</v>
+        <v>30</v>
       </c>
       <c r="G250" s="11">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H250" s="11"/>
       <c r="I250" s="11">
@@ -14324,7 +14318,7 @@
         <v>0</v>
       </c>
       <c r="N250" s="11" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="O250" s="12">
         <f t="shared" si="14"/>
@@ -14341,11 +14335,11 @@
       <c r="V250" s="5"/>
     </row>
     <row r="251" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A251" s="2">
+      <c r="A251" s="36">
         <v>242</v>
       </c>
       <c r="B251" s="11" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C251" s="2" t="s">
         <v>27</v>
@@ -14357,10 +14351,10 @@
         <v>29</v>
       </c>
       <c r="F251" s="2" t="s">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="G251" s="11">
-        <v>108</v>
+        <v>5</v>
       </c>
       <c r="H251" s="11"/>
       <c r="I251" s="11">
@@ -14375,7 +14369,7 @@
         <v>0</v>
       </c>
       <c r="N251" s="11" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="O251" s="12">
         <f t="shared" si="14"/>
@@ -14392,24 +14386,26 @@
       <c r="V251" s="5"/>
     </row>
     <row r="252" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A252" s="2">
+      <c r="A252" s="36">
         <v>243</v>
       </c>
       <c r="B252" s="11" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C252" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D252" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="D252" s="2" t="s">
+        <v>67</v>
+      </c>
       <c r="E252" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F252" s="2" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="G252" s="11">
-        <v>1</v>
+        <v>108</v>
       </c>
       <c r="H252" s="11"/>
       <c r="I252" s="11">
@@ -14424,7 +14420,7 @@
         <v>0</v>
       </c>
       <c r="N252" s="11" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="O252" s="12">
         <f t="shared" si="14"/>
@@ -14441,23 +14437,24 @@
       <c r="V252" s="5"/>
     </row>
     <row r="253" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A253" s="2">
+      <c r="A253" s="36">
         <v>244</v>
       </c>
       <c r="B253" s="11" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C253" s="2" t="s">
-        <v>27</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="D253" s="2"/>
       <c r="E253" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F253" s="2" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="G253" s="11">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="H253" s="11"/>
       <c r="I253" s="11">
@@ -14472,7 +14469,7 @@
         <v>0</v>
       </c>
       <c r="N253" s="11" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="O253" s="12">
         <f t="shared" si="14"/>
@@ -14489,26 +14486,23 @@
       <c r="V253" s="5"/>
     </row>
     <row r="254" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A254" s="2">
+      <c r="A254" s="36">
         <v>245</v>
       </c>
       <c r="B254" s="11" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C254" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D254" s="2" t="s">
-        <v>260</v>
-      </c>
       <c r="E254" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F254" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="G254" s="11">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="H254" s="11"/>
       <c r="I254" s="11">
@@ -14522,8 +14516,8 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="N254" s="15" t="s">
-        <v>360</v>
+      <c r="N254" s="11" t="s">
+        <v>31</v>
       </c>
       <c r="O254" s="12">
         <f t="shared" si="14"/>
@@ -14540,26 +14534,26 @@
       <c r="V254" s="5"/>
     </row>
     <row r="255" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A255" s="2">
+      <c r="A255" s="36">
         <v>246</v>
       </c>
       <c r="B255" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C255" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D255" s="2" t="s">
-        <v>67</v>
+        <v>260</v>
       </c>
       <c r="E255" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F255" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G255" s="11">
-        <v>1</v>
+        <v>64</v>
       </c>
       <c r="H255" s="11"/>
       <c r="I255" s="11">
@@ -14573,14 +14567,16 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="N255" s="11" t="s">
-        <v>50</v>
+      <c r="N255" s="15" t="s">
+        <v>360</v>
       </c>
       <c r="O255" s="12">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P255" s="13"/>
+      <c r="P255" s="13">
+        <v>0</v>
+      </c>
       <c r="Q255" s="14"/>
       <c r="R255" s="14"/>
       <c r="S255" s="14"/>
@@ -14589,11 +14585,11 @@
       <c r="V255" s="5"/>
     </row>
     <row r="256" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A256" s="2">
+      <c r="A256" s="36">
         <v>247</v>
       </c>
       <c r="B256" s="11" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C256" s="2" t="s">
         <v>27</v>
@@ -14608,7 +14604,7 @@
         <v>30</v>
       </c>
       <c r="G256" s="11">
-        <v>59</v>
+        <v>1</v>
       </c>
       <c r="H256" s="11"/>
       <c r="I256" s="11">
@@ -14623,15 +14619,13 @@
         <v>0</v>
       </c>
       <c r="N256" s="11" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="O256" s="12">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P256" s="13">
-        <v>0</v>
-      </c>
+      <c r="P256" s="13"/>
       <c r="Q256" s="14"/>
       <c r="R256" s="14"/>
       <c r="S256" s="14"/>
@@ -14640,11 +14634,11 @@
       <c r="V256" s="5"/>
     </row>
     <row r="257" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A257" s="2">
+      <c r="A257" s="36">
         <v>248</v>
       </c>
       <c r="B257" s="11" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C257" s="2" t="s">
         <v>27</v>
@@ -14659,14 +14653,14 @@
         <v>30</v>
       </c>
       <c r="G257" s="11">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H257" s="11"/>
       <c r="I257" s="11">
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
-      <c r="J257" s="24"/>
+      <c r="J257" s="2"/>
       <c r="K257" s="2"/>
       <c r="L257" s="11"/>
       <c r="M257" s="11">
@@ -14691,11 +14685,11 @@
       <c r="V257" s="5"/>
     </row>
     <row r="258" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A258" s="2">
+      <c r="A258" s="36">
         <v>249</v>
       </c>
       <c r="B258" s="11" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C258" s="2" t="s">
         <v>27</v>
@@ -14707,10 +14701,10 @@
         <v>29</v>
       </c>
       <c r="F258" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="G258" s="11">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="H258" s="11"/>
       <c r="I258" s="11">
@@ -14725,7 +14719,7 @@
         <v>0</v>
       </c>
       <c r="N258" s="11" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="O258" s="12">
         <f t="shared" si="14"/>
@@ -14742,11 +14736,11 @@
       <c r="V258" s="5"/>
     </row>
     <row r="259" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A259" s="2">
+      <c r="A259" s="36">
         <v>250</v>
       </c>
       <c r="B259" s="11" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C259" s="2" t="s">
         <v>27</v>
@@ -14758,10 +14752,10 @@
         <v>29</v>
       </c>
       <c r="F259" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G259" s="11">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="H259" s="11"/>
       <c r="I259" s="11">
@@ -14776,7 +14770,7 @@
         <v>0</v>
       </c>
       <c r="N259" s="11" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="O259" s="12">
         <f t="shared" si="14"/>
@@ -14793,11 +14787,11 @@
       <c r="V259" s="5"/>
     </row>
     <row r="260" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A260" s="2">
+      <c r="A260" s="36">
         <v>251</v>
       </c>
       <c r="B260" s="11" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C260" s="2" t="s">
         <v>27</v>
@@ -14809,10 +14803,10 @@
         <v>29</v>
       </c>
       <c r="F260" s="2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="G260" s="11">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="H260" s="11"/>
       <c r="I260" s="11">
@@ -14827,7 +14821,7 @@
         <v>0</v>
       </c>
       <c r="N260" s="11" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="O260" s="12">
         <f t="shared" si="14"/>
@@ -14844,11 +14838,11 @@
       <c r="V260" s="5"/>
     </row>
     <row r="261" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A261" s="2">
+      <c r="A261" s="36">
         <v>252</v>
       </c>
       <c r="B261" s="11" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C261" s="2" t="s">
         <v>27</v>
@@ -14860,10 +14854,10 @@
         <v>29</v>
       </c>
       <c r="F261" s="2" t="s">
-        <v>150</v>
+        <v>30</v>
       </c>
       <c r="G261" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H261" s="11"/>
       <c r="I261" s="11">
@@ -14895,26 +14889,26 @@
       <c r="V261" s="5"/>
     </row>
     <row r="262" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A262" s="2">
+      <c r="A262" s="36">
         <v>253</v>
       </c>
       <c r="B262" s="11" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C262" s="2" t="s">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="D262" s="2" t="s">
-        <v>255</v>
+        <v>67</v>
       </c>
       <c r="E262" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F262" s="2" t="s">
-        <v>34</v>
+        <v>150</v>
       </c>
       <c r="G262" s="11">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="H262" s="11"/>
       <c r="I262" s="11">
@@ -14928,8 +14922,8 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="N262" s="15" t="s">
-        <v>369</v>
+      <c r="N262" s="11" t="s">
+        <v>50</v>
       </c>
       <c r="O262" s="12">
         <f t="shared" si="14"/>
@@ -14946,29 +14940,30 @@
       <c r="V262" s="5"/>
     </row>
     <row r="263" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A263" s="2">
+      <c r="A263" s="36">
         <v>254</v>
       </c>
       <c r="B263" s="11" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C263" s="2" t="s">
-        <v>27</v>
+        <v>73</v>
       </c>
       <c r="D263" s="2" t="s">
-        <v>67</v>
+        <v>255</v>
       </c>
       <c r="E263" s="2" t="s">
-        <v>348</v>
+        <v>29</v>
       </c>
       <c r="F263" s="2" t="s">
         <v>34</v>
       </c>
       <c r="G263" s="11">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="H263" s="11"/>
       <c r="I263" s="11">
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="J263" s="24"/>
@@ -14978,8 +14973,8 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="N263" s="11" t="s">
-        <v>50</v>
+      <c r="N263" s="15" t="s">
+        <v>369</v>
       </c>
       <c r="O263" s="12">
         <f t="shared" si="14"/>
@@ -14996,11 +14991,11 @@
       <c r="V263" s="5"/>
     </row>
     <row r="264" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A264" s="2">
+      <c r="A264" s="36">
         <v>255</v>
       </c>
       <c r="B264" s="11" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C264" s="2" t="s">
         <v>27</v>
@@ -15009,17 +15004,16 @@
         <v>67</v>
       </c>
       <c r="E264" s="2" t="s">
-        <v>29</v>
+        <v>348</v>
       </c>
       <c r="F264" s="2" t="s">
-        <v>150</v>
+        <v>34</v>
       </c>
       <c r="G264" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H264" s="11"/>
       <c r="I264" s="11">
-        <f t="shared" ref="I264:I271" si="17">H264-J264</f>
         <v>0</v>
       </c>
       <c r="J264" s="24"/>
@@ -15030,7 +15024,7 @@
         <v>0</v>
       </c>
       <c r="N264" s="11" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="O264" s="12">
         <f t="shared" si="14"/>
@@ -15047,68 +15041,68 @@
       <c r="V264" s="5"/>
     </row>
     <row r="265" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A265" s="2">
+      <c r="A265" s="36">
         <v>256</v>
       </c>
-      <c r="B265" s="3" t="s">
-        <v>372</v>
+      <c r="B265" s="11" t="s">
+        <v>371</v>
       </c>
       <c r="C265" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D265" s="2" t="s">
-        <v>373</v>
+        <v>67</v>
       </c>
       <c r="E265" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F265" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="G265" s="3">
-        <v>1</v>
-      </c>
-      <c r="H265" s="3"/>
+        <v>150</v>
+      </c>
+      <c r="G265" s="11">
+        <v>2</v>
+      </c>
+      <c r="H265" s="11"/>
       <c r="I265" s="11">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="J265" s="3"/>
-      <c r="K265" s="3"/>
-      <c r="L265" s="3"/>
+        <f t="shared" ref="I265:I272" si="17">H265-J265</f>
+        <v>0</v>
+      </c>
+      <c r="J265" s="24"/>
+      <c r="K265" s="2"/>
+      <c r="L265" s="11"/>
       <c r="M265" s="11">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="N265" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="O265" s="3">
+        <v>44</v>
+      </c>
+      <c r="O265" s="12">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P265" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q265" s="3"/>
-      <c r="R265" s="3"/>
-      <c r="S265" s="3"/>
-      <c r="T265" s="3"/>
+      <c r="P265" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q265" s="14"/>
+      <c r="R265" s="14"/>
+      <c r="S265" s="14"/>
+      <c r="T265" s="14"/>
       <c r="U265" s="14"/>
       <c r="V265" s="5"/>
     </row>
     <row r="266" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A266" s="2">
+      <c r="A266" s="36">
         <v>257</v>
       </c>
       <c r="B266" s="3" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C266" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D266" s="2" t="s">
-        <v>67</v>
+        <v>373</v>
       </c>
       <c r="E266" s="2" t="s">
         <v>29</v>
@@ -15117,7 +15111,7 @@
         <v>38</v>
       </c>
       <c r="G266" s="3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H266" s="3"/>
       <c r="I266" s="11">
@@ -15126,7 +15120,7 @@
       </c>
       <c r="J266" s="3"/>
       <c r="K266" s="3"/>
-      <c r="L266" s="25"/>
+      <c r="L266" s="3"/>
       <c r="M266" s="11">
         <f t="shared" si="13"/>
         <v>0</v>
@@ -15138,22 +15132,22 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P266" s="25">
-        <v>0</v>
-      </c>
-      <c r="Q266" s="25"/>
-      <c r="R266" s="25"/>
-      <c r="S266" s="25"/>
-      <c r="T266" s="25"/>
+      <c r="P266" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q266" s="3"/>
+      <c r="R266" s="3"/>
+      <c r="S266" s="3"/>
+      <c r="T266" s="3"/>
       <c r="U266" s="14"/>
       <c r="V266" s="5"/>
     </row>
     <row r="267" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A267" s="2">
+      <c r="A267" s="36">
         <v>258</v>
       </c>
       <c r="B267" s="3" t="s">
-        <v>389</v>
+        <v>374</v>
       </c>
       <c r="C267" s="2" t="s">
         <v>27</v>
@@ -15165,10 +15159,10 @@
         <v>29</v>
       </c>
       <c r="F267" s="2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="G267" s="3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H267" s="3"/>
       <c r="I267" s="11">
@@ -15183,7 +15177,7 @@
         <v>0</v>
       </c>
       <c r="N267" s="11" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="O267" s="3">
         <f t="shared" si="14"/>
@@ -15200,11 +15194,11 @@
       <c r="V267" s="5"/>
     </row>
     <row r="268" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A268" s="2">
+      <c r="A268" s="36">
         <v>259</v>
       </c>
       <c r="B268" s="3" t="s">
-        <v>375</v>
+        <v>389</v>
       </c>
       <c r="C268" s="2" t="s">
         <v>27</v>
@@ -15219,7 +15213,7 @@
         <v>30</v>
       </c>
       <c r="G268" s="3">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="H268" s="3"/>
       <c r="I268" s="11">
@@ -15228,34 +15222,34 @@
       </c>
       <c r="J268" s="3"/>
       <c r="K268" s="3"/>
-      <c r="L268" s="3"/>
+      <c r="L268" s="25"/>
       <c r="M268" s="11">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="N268" s="11" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="O268" s="3">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P268" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q268" s="3"/>
-      <c r="R268" s="3"/>
-      <c r="S268" s="3"/>
-      <c r="T268" s="3"/>
-      <c r="U268" s="3"/>
+      <c r="P268" s="25">
+        <v>0</v>
+      </c>
+      <c r="Q268" s="25"/>
+      <c r="R268" s="25"/>
+      <c r="S268" s="25"/>
+      <c r="T268" s="25"/>
+      <c r="U268" s="14"/>
       <c r="V268" s="5"/>
     </row>
     <row r="269" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A269" s="2">
+      <c r="A269" s="36">
         <v>260</v>
       </c>
       <c r="B269" s="3" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C269" s="2" t="s">
         <v>27</v>
@@ -15270,7 +15264,7 @@
         <v>30</v>
       </c>
       <c r="G269" s="3">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="H269" s="3"/>
       <c r="I269" s="11">
@@ -15281,11 +15275,11 @@
       <c r="K269" s="3"/>
       <c r="L269" s="3"/>
       <c r="M269" s="11">
-        <f t="shared" ref="M269:M273" si="18">L269</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="N269" s="11" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="O269" s="3">
         <f t="shared" si="14"/>
@@ -15294,31 +15288,31 @@
       <c r="P269" s="3">
         <v>0</v>
       </c>
-      <c r="Q269" s="25"/>
-      <c r="R269" s="25"/>
-      <c r="S269" s="25"/>
-      <c r="T269" s="25"/>
-      <c r="U269" s="25"/>
+      <c r="Q269" s="3"/>
+      <c r="R269" s="3"/>
+      <c r="S269" s="3"/>
+      <c r="T269" s="3"/>
+      <c r="U269" s="3"/>
       <c r="V269" s="5"/>
     </row>
     <row r="270" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A270" s="2">
+      <c r="A270" s="36">
         <v>261</v>
       </c>
       <c r="B270" s="3" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C270" s="2" t="s">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="D270" s="2" t="s">
-        <v>255</v>
+        <v>67</v>
       </c>
       <c r="E270" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F270" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="G270" s="3">
         <v>1</v>
@@ -15329,20 +15323,20 @@
         <v>0</v>
       </c>
       <c r="J270" s="3"/>
-      <c r="K270" s="25"/>
-      <c r="L270" s="25"/>
+      <c r="K270" s="3"/>
+      <c r="L270" s="3"/>
       <c r="M270" s="11">
-        <f t="shared" si="18"/>
-        <v>0</v>
-      </c>
-      <c r="N270" s="12" t="s">
-        <v>50</v>
+        <f t="shared" ref="M270:M274" si="18">L270</f>
+        <v>0</v>
+      </c>
+      <c r="N270" s="11" t="s">
+        <v>44</v>
       </c>
       <c r="O270" s="3">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P270" s="25">
+      <c r="P270" s="3">
         <v>0</v>
       </c>
       <c r="Q270" s="25"/>
@@ -15353,11 +15347,11 @@
       <c r="V270" s="5"/>
     </row>
     <row r="271" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A271" s="2">
+      <c r="A271" s="36">
         <v>262</v>
       </c>
       <c r="B271" s="3" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C271" s="2" t="s">
         <v>73</v>
@@ -15404,23 +15398,36 @@
       <c r="V271" s="5"/>
     </row>
     <row r="272" spans="1:22" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A272" s="2"/>
-      <c r="B272" s="3"/>
-      <c r="C272" s="2"/>
-      <c r="D272" s="2"/>
-      <c r="E272" s="2"/>
-      <c r="F272" s="2"/>
-      <c r="G272" s="3"/>
-      <c r="H272" s="3">
-        <v>0</v>
-      </c>
-      <c r="I272" s="3"/>
+      <c r="A272" s="36">
+        <v>263</v>
+      </c>
+      <c r="B272" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="C272" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D272" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="E272" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F272" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G272" s="3">
+        <v>1</v>
+      </c>
+      <c r="H272" s="3"/>
+      <c r="I272" s="11">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
       <c r="J272" s="3"/>
-      <c r="K272" s="25" t="s">
-        <v>379</v>
-      </c>
+      <c r="K272" s="25"/>
       <c r="L272" s="25"/>
-      <c r="M272" s="12">
+      <c r="M272" s="11">
         <f t="shared" si="18"/>
         <v>0</v>
       </c>
@@ -15431,193 +15438,204 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P272" s="26">
-        <v>0</v>
-      </c>
-      <c r="Q272" s="26"/>
-      <c r="R272" s="26"/>
-      <c r="S272" s="26"/>
-      <c r="T272" s="26"/>
-      <c r="U272" s="23"/>
-    </row>
-    <row r="273" spans="1:27" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A273" s="38" t="s">
+      <c r="P272" s="25">
+        <v>0</v>
+      </c>
+      <c r="Q272" s="25"/>
+      <c r="R272" s="25"/>
+      <c r="S272" s="25"/>
+      <c r="T272" s="25"/>
+      <c r="U272" s="25"/>
+      <c r="V272" s="5"/>
+    </row>
+    <row r="273" spans="1:27" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A273" s="2"/>
+      <c r="B273" s="3"/>
+      <c r="C273" s="2"/>
+      <c r="D273" s="2"/>
+      <c r="E273" s="2"/>
+      <c r="F273" s="2"/>
+      <c r="G273" s="3"/>
+      <c r="H273" s="3">
+        <v>0</v>
+      </c>
+      <c r="I273" s="3"/>
+      <c r="J273" s="3"/>
+      <c r="K273" s="25" t="s">
+        <v>379</v>
+      </c>
+      <c r="L273" s="25"/>
+      <c r="M273" s="12">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="N273" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="O273" s="3">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="P273" s="26">
+        <v>0</v>
+      </c>
+      <c r="Q273" s="26"/>
+      <c r="R273" s="26"/>
+      <c r="S273" s="26"/>
+      <c r="T273" s="26"/>
+      <c r="U273" s="23"/>
+    </row>
+    <row r="274" spans="1:27" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A274" s="43" t="s">
         <v>380</v>
       </c>
-      <c r="B273" s="38"/>
-      <c r="C273" s="38"/>
-      <c r="D273" s="38"/>
-      <c r="E273" s="38"/>
-      <c r="F273" s="38"/>
-      <c r="G273" s="38"/>
-      <c r="H273" s="38"/>
-      <c r="I273" s="38"/>
-      <c r="J273" s="38"/>
-      <c r="K273" s="38"/>
-      <c r="L273" s="11"/>
-      <c r="M273" s="11">
+      <c r="B274" s="43"/>
+      <c r="C274" s="43"/>
+      <c r="D274" s="43"/>
+      <c r="E274" s="43"/>
+      <c r="F274" s="43"/>
+      <c r="G274" s="43"/>
+      <c r="H274" s="43"/>
+      <c r="I274" s="43"/>
+      <c r="J274" s="43"/>
+      <c r="K274" s="43"/>
+      <c r="L274" s="11"/>
+      <c r="M274" s="11">
         <f t="shared" si="18"/>
         <v>0</v>
       </c>
-      <c r="N273" s="11"/>
-      <c r="O273" s="11"/>
-      <c r="P273" s="27"/>
-      <c r="Q273" s="14"/>
-      <c r="R273" s="14"/>
-      <c r="S273" s="14"/>
-      <c r="T273" s="14"/>
-      <c r="U273" s="19"/>
-      <c r="V273" s="5"/>
-    </row>
-    <row r="274" spans="1:27" s="30" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A274" s="28"/>
-      <c r="B274" s="29" t="s">
+      <c r="N274" s="11"/>
+      <c r="O274" s="11"/>
+      <c r="P274" s="27"/>
+      <c r="Q274" s="14"/>
+      <c r="R274" s="14"/>
+      <c r="S274" s="14"/>
+      <c r="T274" s="14"/>
+      <c r="U274" s="19"/>
+      <c r="V274" s="5"/>
+    </row>
+    <row r="275" spans="1:27" s="30" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A275" s="28"/>
+      <c r="B275" s="29" t="s">
         <v>381</v>
       </c>
-      <c r="C274" s="28"/>
-      <c r="D274" s="28"/>
-      <c r="E274" s="28"/>
-      <c r="F274" s="8"/>
-      <c r="G274" s="28">
-        <f>SUM(G10:G271)</f>
-        <v>22283</v>
-      </c>
-      <c r="H274" s="28">
-        <f>SUM(H10:H271)</f>
-        <v>0</v>
-      </c>
-      <c r="I274" s="28">
-        <f>SUM(I10:I271)</f>
-        <v>0</v>
-      </c>
-      <c r="J274" s="28">
-        <f>SUM(J10:J271)</f>
-        <v>0</v>
-      </c>
-      <c r="K274" s="28">
-        <f>SUM(K10:K271)</f>
-        <v>0</v>
-      </c>
-      <c r="L274" s="28">
-        <f>SUM(L10:L273)</f>
-        <v>0</v>
-      </c>
-      <c r="M274" s="28">
-        <f>SUM(M10:M273)</f>
-        <v>0</v>
-      </c>
-      <c r="N274" s="8"/>
-      <c r="O274" s="28">
-        <f>SUM(O10:O273)-L273</f>
-        <v>0</v>
-      </c>
-      <c r="P274" s="28">
-        <f>SUM(P10:P273)</f>
-        <v>0</v>
-      </c>
-      <c r="Q274" s="28">
-        <f>SUM(Q10:Q273)</f>
-        <v>0</v>
-      </c>
-      <c r="R274" s="28">
-        <f>SUM(R10:R273)</f>
-        <v>0</v>
-      </c>
-      <c r="S274" s="28">
-        <f>SUM(S10:S273)</f>
-        <v>0</v>
-      </c>
-      <c r="T274" s="28">
-        <f>SUM(T10:T273)</f>
-        <v>0</v>
-      </c>
-      <c r="U274" s="28"/>
-    </row>
-    <row r="275" spans="1:27" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B275" s="31" t="s">
-        <v>382</v>
-      </c>
-      <c r="G275" s="32" t="s">
-        <v>383</v>
-      </c>
-      <c r="H275" s="33">
-        <f>H272+I274+J274</f>
-        <v>0</v>
-      </c>
-      <c r="I275" s="18"/>
-      <c r="M275" s="18"/>
+      <c r="C275" s="28"/>
+      <c r="D275" s="28"/>
+      <c r="E275" s="28"/>
+      <c r="F275" s="8"/>
+      <c r="G275" s="28">
+        <f>SUM(G10:G272)</f>
+        <v>22284</v>
+      </c>
+      <c r="H275" s="28">
+        <f>SUM(H10:H272)</f>
+        <v>0</v>
+      </c>
+      <c r="I275" s="28">
+        <f>SUM(I10:I272)</f>
+        <v>0</v>
+      </c>
+      <c r="J275" s="28">
+        <f>SUM(J10:J272)</f>
+        <v>0</v>
+      </c>
+      <c r="K275" s="28">
+        <f>SUM(K10:K272)</f>
+        <v>0</v>
+      </c>
+      <c r="L275" s="28">
+        <f>SUM(L10:L274)</f>
+        <v>0</v>
+      </c>
+      <c r="M275" s="28">
+        <f>SUM(M10:M274)</f>
+        <v>0</v>
+      </c>
+      <c r="N275" s="8"/>
+      <c r="O275" s="28">
+        <f>SUM(O10:O274)-L274</f>
+        <v>0</v>
+      </c>
+      <c r="P275" s="28">
+        <f>SUM(P10:P274)</f>
+        <v>0</v>
+      </c>
+      <c r="Q275" s="28">
+        <f>SUM(Q10:Q274)</f>
+        <v>0</v>
+      </c>
+      <c r="R275" s="28">
+        <f>SUM(R10:R274)</f>
+        <v>0</v>
+      </c>
+      <c r="S275" s="28">
+        <f>SUM(S10:S274)</f>
+        <v>0</v>
+      </c>
+      <c r="T275" s="28">
+        <f>SUM(T10:T274)</f>
+        <v>0</v>
+      </c>
+      <c r="U275" s="28"/>
     </row>
     <row r="276" spans="1:27" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B276" s="31" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="G276" s="32" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="H276" s="33">
-        <f>H275+P274</f>
+        <f>H273+I275+J275</f>
         <v>0</v>
       </c>
       <c r="I276" s="18"/>
       <c r="M276" s="18"/>
     </row>
-    <row r="278" spans="1:27" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A278" s="34"/>
-      <c r="B278" s="34"/>
-      <c r="C278" s="34"/>
-      <c r="D278" s="34"/>
-      <c r="E278" s="34"/>
-      <c r="F278" s="34"/>
-      <c r="G278" s="34"/>
-      <c r="H278" s="36" t="s">
+    <row r="277" spans="1:27" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B277" s="31" t="s">
+        <v>384</v>
+      </c>
+      <c r="G277" s="32" t="s">
+        <v>385</v>
+      </c>
+      <c r="H277" s="33">
+        <f>H276+P275</f>
+        <v>0</v>
+      </c>
+      <c r="I277" s="18"/>
+      <c r="M277" s="18"/>
+    </row>
+    <row r="279" spans="1:27" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A279" s="34"/>
+      <c r="B279" s="34"/>
+      <c r="C279" s="34"/>
+      <c r="D279" s="34"/>
+      <c r="E279" s="34"/>
+      <c r="F279" s="34"/>
+      <c r="G279" s="34"/>
+      <c r="H279" s="42" t="s">
         <v>386</v>
       </c>
-      <c r="I278" s="36"/>
-      <c r="J278" s="36"/>
-      <c r="K278" s="36"/>
-      <c r="L278" s="36"/>
-      <c r="M278" s="36"/>
-      <c r="N278" s="36"/>
-      <c r="O278" s="36"/>
-      <c r="P278" s="36"/>
-      <c r="Q278" s="36"/>
-      <c r="R278" s="36"/>
-      <c r="S278" s="34"/>
-      <c r="T278" s="34"/>
-      <c r="U278" s="34"/>
-      <c r="V278" s="34"/>
-      <c r="W278" s="34"/>
-      <c r="X278" s="34"/>
-      <c r="Y278" s="34"/>
-      <c r="Z278" s="34"/>
-      <c r="AA278" s="34"/>
-    </row>
-    <row r="279" spans="1:27" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A279" s="35"/>
-      <c r="B279" s="35"/>
-      <c r="C279" s="35"/>
-      <c r="D279" s="35"/>
-      <c r="E279" s="35"/>
-      <c r="F279" s="35"/>
-      <c r="G279" s="35"/>
-      <c r="H279" s="35"/>
-      <c r="I279" s="35"/>
-      <c r="J279" s="35"/>
-      <c r="K279" s="35"/>
-      <c r="L279" s="35"/>
-      <c r="M279" s="35"/>
-      <c r="N279" s="35"/>
-      <c r="O279" s="35"/>
-      <c r="P279" s="35"/>
-      <c r="Q279" s="35"/>
-      <c r="R279" s="35"/>
-      <c r="S279" s="35"/>
-      <c r="T279" s="35"/>
-      <c r="U279" s="35"/>
-      <c r="V279" s="35"/>
-      <c r="W279" s="35"/>
-      <c r="X279" s="35"/>
-      <c r="Y279" s="35"/>
+      <c r="I279" s="42"/>
+      <c r="J279" s="42"/>
+      <c r="K279" s="42"/>
+      <c r="L279" s="42"/>
+      <c r="M279" s="42"/>
+      <c r="N279" s="42"/>
+      <c r="O279" s="42"/>
+      <c r="P279" s="42"/>
+      <c r="Q279" s="42"/>
+      <c r="R279" s="42"/>
+      <c r="S279" s="34"/>
+      <c r="T279" s="34"/>
+      <c r="U279" s="34"/>
+      <c r="V279" s="34"/>
+      <c r="W279" s="34"/>
+      <c r="X279" s="34"/>
+      <c r="Y279" s="34"/>
+      <c r="Z279" s="34"/>
+      <c r="AA279" s="34"/>
     </row>
     <row r="280" spans="1:27" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A280" s="35"/>
@@ -15646,8 +15664,46 @@
       <c r="X280" s="35"/>
       <c r="Y280" s="35"/>
     </row>
+    <row r="281" spans="1:27" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A281" s="35"/>
+      <c r="B281" s="35"/>
+      <c r="C281" s="35"/>
+      <c r="D281" s="35"/>
+      <c r="E281" s="35"/>
+      <c r="F281" s="35"/>
+      <c r="G281" s="35"/>
+      <c r="H281" s="35"/>
+      <c r="I281" s="35"/>
+      <c r="J281" s="35"/>
+      <c r="K281" s="35"/>
+      <c r="L281" s="35"/>
+      <c r="M281" s="35"/>
+      <c r="N281" s="35"/>
+      <c r="O281" s="35"/>
+      <c r="P281" s="35"/>
+      <c r="Q281" s="35"/>
+      <c r="R281" s="35"/>
+      <c r="S281" s="35"/>
+      <c r="T281" s="35"/>
+      <c r="U281" s="35"/>
+      <c r="V281" s="35"/>
+      <c r="W281" s="35"/>
+      <c r="X281" s="35"/>
+      <c r="Y281" s="35"/>
+    </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="H279:R279"/>
+    <mergeCell ref="M7:M8"/>
+    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="Q7:R7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="A274:K274"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="L7:L8"/>
     <mergeCell ref="T1:U3"/>
     <mergeCell ref="A4:U4"/>
     <mergeCell ref="A6:A8"/>
@@ -15664,25 +15720,14 @@
     <mergeCell ref="D7:D8"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="F7:F8"/>
-    <mergeCell ref="H278:R278"/>
-    <mergeCell ref="M7:M8"/>
-    <mergeCell ref="N7:N8"/>
-    <mergeCell ref="Q7:R7"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="A273:K273"/>
-    <mergeCell ref="H7:H8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="K7:K8"/>
-    <mergeCell ref="L7:L8"/>
   </mergeCells>
-  <conditionalFormatting sqref="B147:B264 B272 B10:B143">
+  <conditionalFormatting sqref="B147:B265 B273 B10:B143">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" scale="10" firstPageNumber="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="274" max="16383" man="1"/>
+    <brk id="275" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>